<commit_message>
Fix synthesis table localization and merged cells
</commit_message>
<xml_diff>
--- a/source/downloads/skill-magic-synthesis.xlsx
+++ b/source/downloads/skill-magic-synthesis.xlsx
@@ -58,7 +58,7 @@
     <t>雅</t>
   </si>
   <si>
-    <t>備考</t>
+    <t>备注</t>
   </si>
   <si>
     <t>最终破击</t>
@@ -433,13 +433,13 @@
     <t>缩小</t>
   </si>
   <si>
-    <t>テ</t>
-  </si>
-  <si>
-    <t>ヴ</t>
-  </si>
-  <si>
-    <t>ア</t>
+    <t>泰</t>
+  </si>
+  <si>
+    <t>维</t>
+  </si>
+  <si>
+    <t>雅</t>
   </si>
   <si>
     <t>连击滑行</t>
@@ -4122,7 +4122,7 @@
       <c r="H109" s="13"/>
     </row>
   </sheetData>
-  <mergeCells count="202">
+  <mergeCells count="204">
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="A7:A8"/>
@@ -4158,7 +4158,9 @@
     <mergeCell ref="A106:A109"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="B9:B10"/>
+    <mergeCell ref="B12:B13"/>
     <mergeCell ref="B16:B17"/>
+    <mergeCell ref="B19:B20"/>
     <mergeCell ref="B24:B25"/>
     <mergeCell ref="B26:B27"/>
     <mergeCell ref="B28:B29"/>

</xml_diff>